<commit_message>
Changed names from English to Hebrew
</commit_message>
<xml_diff>
--- a/G1_Assigment1/G1_Acceptance.Ass1.xlsx
+++ b/G1_Assigment1/G1_Acceptance.Ass1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almo1\GoNature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almo1\Desktop\G1_Assigment1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{999B5D02-585E-4DB6-9575-AC4FB9226558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5DABBC-8B3F-40BC-807B-265962615A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{66F18C86-3E6B-4F2E-A3A6-956843228F2B}"/>
   </bookViews>
@@ -1842,11 +1842,11 @@
   </si>
   <si>
     <t>Group #1, members: 
-Bar Sagi, bar.sagi@e.braude.ac.il
-Shiraz Shamai, shiraz.shamai@e.braude.ac.il
-Gal Dolev, gal.dolev@e.braude.ac.il
-Reut Dahan, reut.dahan@e.braude.ac.il
-date: 09/04/2026</t>
+בר שגיא, bar.sagi@e.braude.ac.il
+שירז שמאי, shiraz.shamai@e.braude.ac.il
+גל דולב, gal.dolev@e.braude.ac.il
+רעות דהן, reut.dahan@e.braude.ac.il
+date: 10/04/2026</t>
   </si>
 </sst>
 </file>
@@ -2007,10 +2007,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2026,10 +2022,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2359,8 +2359,8 @@
     <col min="3" max="3" width="5.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="9" customFormat="1" ht="93.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:3" s="15" customFormat="1" ht="93.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>257</v>
       </c>
     </row>
@@ -3269,33 +3269,33 @@
   <dimension ref="A1:E80"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="79.75" style="14" customWidth="1"/>
-    <col min="2" max="2" width="36.875" style="11" customWidth="1"/>
-    <col min="3" max="3" width="39.125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="38.625" style="11" customWidth="1"/>
-    <col min="5" max="5" width="47.125" style="11" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="11"/>
+    <col min="1" max="1" width="79.75" style="12" customWidth="1"/>
+    <col min="2" max="2" width="36.875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="39.125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="38.625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="47.125" style="9" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="15" customFormat="1" ht="96.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:5" s="16" customFormat="1" ht="96.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>445</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="8" t="s">
         <v>8</v>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="120" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>441</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -3452,7 +3452,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="16" customFormat="1" ht="75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" s="13" customFormat="1" ht="75" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>95</v>
       </c>

</xml_diff>